<commit_message>
feat: split member name into first/last and add hire_date field
Replace single `name` column with `first_name`/`last_name` (NOT NULL)
and add `hire_date` (Date, nullable) across the full stack. Migration
splits existing data via SPLIT_PART and handles single-word names.
Model @property provides backward-compatible computed display name for
tree services and seed output. Update form with separate first/last
name fields and native date picker for hire date. Update all display
components, search filters, import mapper/commit, and tests.

PRP: .context/features/018-member-name-split/PRP.md

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/valid_members.xlsx
+++ b/backend/tests/fixtures/valid_members.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O6"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -424,70 +424,75 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>first_name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
+          <t>last_name</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
           <t>title</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>location</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>slack_handle</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>salary</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>bonus</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>pto_used</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>functional_area_name</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>team_name</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>program_name</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>supervisor_employee_id</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>program_role</t>
         </is>
@@ -501,60 +506,63 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Alice Smith</t>
+          <t>Alice</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Smith</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>New York</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>alice@example.com</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>555-0001</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>@alice</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>120000</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>10000</v>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>5</v>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Backend</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Alpha</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -564,64 +572,68 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bob Jones</t>
+          <t>Bob</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Jones</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Designer</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>London</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>bob@example.com</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>555-0002</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>@bob</t>
         </is>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>95000</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>8000</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>3.5</v>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>UX</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>EMP001</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -631,60 +643,64 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Carol White</t>
+          <t>Carol</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>White</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Chicago</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>carol@example.com</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>555-0003</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>@carol</t>
         </is>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>140000</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>15000</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>2</v>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Backend</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Alpha</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>Lead</t>
         </is>
@@ -698,64 +714,68 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Dave Brown</t>
+          <t>Dave</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Brown</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>Analyst</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Austin</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>dave@example.com</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>555-0004</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>@dave</t>
         </is>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>85000</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>5000</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>8</v>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Analytics</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Gamma</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>EMP003</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -765,64 +785,68 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Eve Davis</t>
+          <t>Eve</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>Davis</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>Engineer</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Seattle</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>eve@example.com</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>555-0005</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>@eve</t>
         </is>
       </c>
-      <c r="H6" t="n">
+      <c r="I6" t="n">
         <v>110000</v>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>9000</v>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="n">
         <v>4.5</v>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Engineering</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Frontend</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Alpha</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>EMP001</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix: update test fixtures to use city/state instead of location
valid_members.csv and .xlsx still had the old location column from
before the city/state split (feature 020). Replace with city + state
columns so the pass-through column maps in 4 tests resolve to valid
target fields. All 170 tests now pass.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/valid_members.xlsx
+++ b/backend/tests/fixtures/valid_members.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:Q6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,60 +439,65 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>city</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>email</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>slack_handle</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>salary</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>bonus</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>pto_used</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>functional_area_name</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>team_name</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>program_name</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>supervisor_employee_id</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>program_role</t>
         </is>
@@ -526,43 +531,56 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>alice@example.com</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>555-0001</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>@alice</t>
         </is>
       </c>
-      <c r="I2" t="n">
-        <v>120000</v>
-      </c>
-      <c r="J2" t="n">
-        <v>10000</v>
-      </c>
-      <c r="K2" t="n">
-        <v>5</v>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>120000</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
           <t>Engineering</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>Backend</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Alpha</t>
         </is>
       </c>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -590,50 +608,58 @@
           <t>London</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr">
         <is>
           <t>bob@example.com</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>555-0002</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>@bob</t>
         </is>
       </c>
-      <c r="I3" t="n">
-        <v>95000</v>
-      </c>
-      <c r="J3" t="n">
-        <v>8000</v>
-      </c>
-      <c r="K3" t="n">
-        <v>3.5</v>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>95000</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>8000</t>
+        </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
+          <t>3.5</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
           <t>Design</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>UX</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
+      <c r="O3" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
+      <c r="P3" t="inlineStr">
         <is>
           <t>EMP001</t>
         </is>
       </c>
+      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -663,44 +689,56 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
+          <t>IL</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>carol@example.com</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>555-0003</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>@carol</t>
         </is>
       </c>
-      <c r="I4" t="n">
-        <v>140000</v>
-      </c>
-      <c r="J4" t="n">
-        <v>15000</v>
-      </c>
-      <c r="K4" t="n">
-        <v>2</v>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>140000</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>15000</t>
+        </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
           <t>Engineering</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Backend</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Alpha</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="P4" t="inlineStr"/>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Lead</t>
         </is>
@@ -734,48 +772,60 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
+          <t>TX</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>dave@example.com</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>555-0004</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>@dave</t>
         </is>
       </c>
-      <c r="I5" t="n">
-        <v>85000</v>
-      </c>
-      <c r="J5" t="n">
-        <v>5000</v>
-      </c>
-      <c r="K5" t="n">
-        <v>8</v>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>85000</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>5000</t>
+        </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
+          <t>8.0</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>Analytics</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>Gamma</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>EMP003</t>
         </is>
       </c>
+      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -805,48 +855,60 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
+          <t>WA</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
           <t>eve@example.com</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>555-0005</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>@eve</t>
         </is>
       </c>
-      <c r="I6" t="n">
-        <v>110000</v>
-      </c>
-      <c r="J6" t="n">
-        <v>9000</v>
-      </c>
-      <c r="K6" t="n">
-        <v>4.5</v>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>110000</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>9000</t>
+        </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
           <t>Engineering</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>Frontend</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
+      <c r="O6" t="inlineStr">
         <is>
           <t>Alpha</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>EMP001</t>
         </is>
       </c>
+      <c r="Q6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: import members into multiple programs (feature 056)
- Add semicolon-delimited program_names + program_team_names import
  fields with positional alignment and length validation
- Apply replace semantics on commit (programs not listed are unassigned),
  guarded so blank/empty cells are no-ops, not mass-deletes
- Two-stage import preview: cheap during mapping iteration, full DB
  diff on entry to PreviewStep so destructive deltas appear before commit
- Eager-load program_assignments + program_team on member list endpoint
- MemberCard +N more overflow chip with team subscript; ProgramTree
  ×N badge for members in multiple programs
- UniqueConstraint on program_teams (program_id, name) with migration
  and IntegrityError-safe get-or-create
- 15 new backend tests, 2 new frontend tests
- Drive-by: fix E402/mypy debt in import_commit.py and
  import_commit_members.py (lint −15, typecheck −6 vs baseline)

PRP: .context/features/056-multi-program-member-import/PRP.md
</commit_message>
<xml_diff>
--- a/backend/tests/fixtures/valid_members.xlsx
+++ b/backend/tests/fixtures/valid_members.xlsx
@@ -489,7 +489,7 @@
       </c>
       <c r="O1" t="inlineStr">
         <is>
-          <t>program_name</t>
+          <t>program_names</t>
         </is>
       </c>
       <c r="P1" t="inlineStr">
@@ -579,8 +579,6 @@
           <t>Alpha</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -608,7 +606,6 @@
           <t>London</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>bob@example.com</t>
@@ -659,7 +656,6 @@
           <t>EMP001</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -737,7 +733,6 @@
           <t>Alpha</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr">
         <is>
           <t>Lead</t>
@@ -825,7 +820,6 @@
           <t>EMP003</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -908,7 +902,6 @@
           <t>EMP001</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>